<commit_message>
Reset Excel Table for MIG CO2-02
</commit_message>
<xml_diff>
--- a/FM-MN-07_MIG CO2-02.xlsx
+++ b/FM-MN-07_MIG CO2-02.xlsx
@@ -1753,17 +1753,9 @@
           <t>ตรวจสภาพความพร้อมโดยรวมของเครื่อง</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C6" s="14" t="inlineStr"/>
       <c r="D6" s="14" t="inlineStr"/>
-      <c r="E6" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr"/>
       <c r="H6" s="14" t="inlineStr"/>
@@ -1802,17 +1794,9 @@
           <t>เช็ค BREAKER เพื่อเช็คระบบไฟฟ้า ตามตำแหน่งไฟ โชว์ และสวิชท์ต่าง ๆ</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C7" s="14" t="inlineStr"/>
       <c r="D7" s="14" t="inlineStr"/>
-      <c r="E7" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr"/>
       <c r="G7" s="14" t="inlineStr"/>
       <c r="H7" s="14" t="inlineStr"/>
@@ -1851,17 +1835,9 @@
           <t>ตรวจสภาพความพร้อมของมาตราวัดแรงดัน ของก๊าซ CO2 และปรับตั้งอย่างถูกต้อง</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C8" s="14" t="inlineStr"/>
       <c r="D8" s="14" t="inlineStr"/>
-      <c r="E8" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
       <c r="G8" s="14" t="inlineStr"/>
       <c r="H8" s="14" t="inlineStr"/>
@@ -1900,17 +1876,9 @@
           <t>ตรวจจุดต่อของก๊าซ CO2 รั่วหรือไม่</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C9" s="14" t="inlineStr"/>
       <c r="D9" s="14" t="inlineStr"/>
-      <c r="E9" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
       <c r="G9" s="14" t="inlineStr"/>
       <c r="H9" s="14" t="inlineStr"/>
@@ -1949,17 +1917,9 @@
           <t>ตรวจสภาพความพร้อมของสายไฟ สายก๊าซ  CO2 ว่ารั่วหรือไม่</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C10" s="14" t="inlineStr"/>
       <c r="D10" s="14" t="inlineStr"/>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
       <c r="G10" s="14" t="inlineStr"/>
       <c r="H10" s="14" t="inlineStr"/>
@@ -1998,17 +1958,9 @@
           <t>ตรวจสภาพความพร้อมของสายกราวด์</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C11" s="14" t="inlineStr"/>
       <c r="D11" s="14" t="inlineStr"/>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
       <c r="G11" s="14" t="inlineStr"/>
       <c r="H11" s="14" t="inlineStr"/>
@@ -2047,17 +1999,9 @@
           <t>ทำความสะอาดหัวเชื่อมก่อนใช้งาน</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr"/>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
+      <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr"/>
       <c r="H12" s="14" t="inlineStr"/>
@@ -2090,17 +2034,9 @@
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="8" t="n"/>
       <c r="B13" s="7" t="n"/>
-      <c r="C13" s="31" t="inlineStr">
-        <is>
-          <t>อินทัช เป็นสุข</t>
-        </is>
-      </c>
+      <c r="C13" s="31" t="inlineStr"/>
       <c r="D13" s="30" t="inlineStr"/>
-      <c r="E13" s="31" t="inlineStr">
-        <is>
-          <t>อินทัช เป็นสุข</t>
-        </is>
-      </c>
+      <c r="E13" s="31" t="inlineStr"/>
       <c r="F13" s="30" t="inlineStr"/>
       <c r="G13" s="30" t="inlineStr"/>
       <c r="H13" s="30" t="inlineStr"/>

</xml_diff>

<commit_message>
Direct Write Excel for MIG CO2-02 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_MIG CO2-02.xlsx
+++ b/FM-MN-07_MIG CO2-02.xlsx
@@ -1758,7 +1758,11 @@
       <c r="E6" s="14" t="inlineStr"/>
       <c r="F6" s="14" t="inlineStr"/>
       <c r="G6" s="14" t="inlineStr"/>
-      <c r="H6" s="14" t="inlineStr"/>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="14" t="inlineStr"/>
       <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr"/>
@@ -1799,7 +1803,11 @@
       <c r="E7" s="14" t="inlineStr"/>
       <c r="F7" s="14" t="inlineStr"/>
       <c r="G7" s="14" t="inlineStr"/>
-      <c r="H7" s="14" t="inlineStr"/>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="14" t="inlineStr"/>
       <c r="J7" s="14" t="inlineStr"/>
       <c r="K7" s="14" t="inlineStr"/>
@@ -1840,7 +1848,11 @@
       <c r="E8" s="14" t="inlineStr"/>
       <c r="F8" s="14" t="inlineStr"/>
       <c r="G8" s="14" t="inlineStr"/>
-      <c r="H8" s="14" t="inlineStr"/>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="14" t="inlineStr"/>
       <c r="J8" s="14" t="inlineStr"/>
       <c r="K8" s="14" t="inlineStr"/>
@@ -1881,7 +1893,11 @@
       <c r="E9" s="14" t="inlineStr"/>
       <c r="F9" s="14" t="inlineStr"/>
       <c r="G9" s="14" t="inlineStr"/>
-      <c r="H9" s="14" t="inlineStr"/>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="14" t="inlineStr"/>
       <c r="J9" s="14" t="inlineStr"/>
       <c r="K9" s="14" t="inlineStr"/>
@@ -1922,7 +1938,11 @@
       <c r="E10" s="14" t="inlineStr"/>
       <c r="F10" s="14" t="inlineStr"/>
       <c r="G10" s="14" t="inlineStr"/>
-      <c r="H10" s="14" t="inlineStr"/>
+      <c r="H10" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="14" t="inlineStr"/>
       <c r="J10" s="14" t="inlineStr"/>
       <c r="K10" s="14" t="inlineStr"/>
@@ -1963,7 +1983,11 @@
       <c r="E11" s="14" t="inlineStr"/>
       <c r="F11" s="14" t="inlineStr"/>
       <c r="G11" s="14" t="inlineStr"/>
-      <c r="H11" s="14" t="inlineStr"/>
+      <c r="H11" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I11" s="14" t="inlineStr"/>
       <c r="J11" s="14" t="inlineStr"/>
       <c r="K11" s="14" t="inlineStr"/>
@@ -2004,7 +2028,11 @@
       <c r="E12" s="14" t="inlineStr"/>
       <c r="F12" s="14" t="inlineStr"/>
       <c r="G12" s="14" t="inlineStr"/>
-      <c r="H12" s="14" t="inlineStr"/>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I12" s="14" t="inlineStr"/>
       <c r="J12" s="14" t="inlineStr"/>
       <c r="K12" s="14" t="inlineStr"/>
@@ -2039,7 +2067,11 @@
       <c r="E13" s="31" t="inlineStr"/>
       <c r="F13" s="30" t="inlineStr"/>
       <c r="G13" s="30" t="inlineStr"/>
-      <c r="H13" s="30" t="inlineStr"/>
+      <c r="H13" s="31" t="inlineStr">
+        <is>
+          <t>อนุสรณ์  ชื่นแฉ่ง</t>
+        </is>
+      </c>
       <c r="I13" s="30" t="inlineStr"/>
       <c r="J13" s="30" t="inlineStr"/>
       <c r="K13" s="30" t="inlineStr"/>
@@ -2176,7 +2208,11 @@
       </c>
     </row>
     <row r="18" ht="338.25" customHeight="1">
-      <c r="B18" s="41" t="inlineStr"/>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>[วันที่ 6]: ข้อ 7: พบปัณไฟไม่สเถียรขณะเชื่อมเดินแนวปรับไฟเชื่อมเดินแนวใด้ไม่สเถียรพบปัณหา 5/8/69  เวลา11:30น. ต้องให้ช่าง  OTC  เข้ามาเช็ค</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="21" customHeight="1">
       <c r="AA19" s="5" t="n"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for MIG CO2-02 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_MIG CO2-02.xlsx
+++ b/FM-MN-07_MIG CO2-02.xlsx
@@ -1763,7 +1763,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J6" s="14" t="inlineStr"/>
       <c r="K6" s="14" t="inlineStr"/>
       <c r="L6" s="14" t="inlineStr"/>
@@ -1808,7 +1812,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="14" t="inlineStr"/>
+      <c r="I7" s="14" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J7" s="14" t="inlineStr"/>
       <c r="K7" s="14" t="inlineStr"/>
       <c r="L7" s="14" t="inlineStr"/>
@@ -1853,7 +1861,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr"/>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="14" t="inlineStr"/>
       <c r="K8" s="14" t="inlineStr"/>
       <c r="L8" s="14" t="inlineStr"/>
@@ -1898,7 +1910,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="14" t="inlineStr"/>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="14" t="inlineStr"/>
       <c r="K9" s="14" t="inlineStr"/>
       <c r="L9" s="14" t="inlineStr"/>
@@ -1943,7 +1959,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="14" t="inlineStr"/>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="14" t="inlineStr"/>
       <c r="K10" s="14" t="inlineStr"/>
       <c r="L10" s="14" t="inlineStr"/>
@@ -1988,7 +2008,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I11" s="14" t="inlineStr"/>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J11" s="14" t="inlineStr"/>
       <c r="K11" s="14" t="inlineStr"/>
       <c r="L11" s="14" t="inlineStr"/>
@@ -2033,7 +2057,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I12" s="14" t="inlineStr"/>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J12" s="14" t="inlineStr"/>
       <c r="K12" s="14" t="inlineStr"/>
       <c r="L12" s="14" t="inlineStr"/>
@@ -2072,7 +2100,11 @@
           <t>อนุสรณ์  ชื่นแฉ่ง</t>
         </is>
       </c>
-      <c r="I13" s="30" t="inlineStr"/>
+      <c r="I13" s="31" t="inlineStr">
+        <is>
+          <t>อนุสรณ์  ชื่นแฉ่ง</t>
+        </is>
+      </c>
       <c r="J13" s="30" t="inlineStr"/>
       <c r="K13" s="30" t="inlineStr"/>
       <c r="L13" s="30" t="inlineStr"/>
@@ -2210,7 +2242,7 @@
     <row r="18" ht="338.25" customHeight="1">
       <c r="B18" s="41" t="inlineStr">
         <is>
-          <t>[วันที่ 6]: ข้อ 7: พบปัณไฟไม่สเถียรขณะเชื่อมเดินแนวปรับไฟเชื่อมเดินแนวใด้ไม่สเถียรพบปัณหา 5/8/69  เวลา11:30น. ต้องให้ช่าง  OTC  เข้ามาเช็ค,  [วันที่ 6]: ข้อ 7: พบปัณไฟไม่สเถียรขณะเชื่อมเดินแนวปรับไฟเชื่อมเดินแนวใด้ไม่สเถียรพบปัณหา 5/8/69  เวลา11:30น. ต้องให้ช่าง  OTC  เข้ามาเช็ค</t>
+          <t>[วันที่ 6]: ข้อ 7: พบปัณไฟไม่สเถียรขณะเชื่อมเดินแนวปรับไฟเชื่อมเดินแนวใด้ไม่สเถียรพบปัณหา 5/8/69  เวลา11:30น. ต้องให้ช่าง  OTC  เข้ามาเช็ค,  [วันที่ 6]: ข้อ 7: พบปัณไฟไม่สเถียรขณะเชื่อมเดินแนวปรับไฟเชื่อมเดินแนวใด้ไม่สเถียรพบปัณหา 5/8/69  เวลา11:30น. ต้องให้ช่าง  OTC  เข้ามาเช็ค,  [วันที่ 7]: ข้อ 1: กระแสไฟไม่สเถียร ระบบรวนเชื่อมเดินแนวไม่ใด้ พบอาการ 5/8/26  เวลา11:30, ข้อ 2: สวิทเปิดไม่ค่อยติดพบอาการ 6/8/26</t>
         </is>
       </c>
     </row>

</xml_diff>